<commit_message>
Update bulk upload sheet — typo fix confirmed on 20% off ad
https://claude.ai/code/session_01KqjHkizaco74VDp8DBP6wH
</commit_message>
<xml_diff>
--- a/ads-strategy/meta-bulk-upload.xlsx
+++ b/ads-strategy/meta-bulk-upload.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,12 @@
       <b val="1"/>
       <color rgb="005D3A1A"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <color rgb="001a7a1a"/>
     </font>
   </fonts>
   <fills count="5">
@@ -85,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -101,6 +107,10 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -804,9 +814,9 @@
           <t>https://parksapparel.com</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ TYPO in image: 'First Tiime' → fix to 'First Time' before running. Confirm HAPPYTRAILS20 code is active in Shopify.</t>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>Typo fixed ✅ — Confirm HAPPYTRAILS20 code is active in Shopify before running</t>
         </is>
       </c>
     </row>
@@ -834,9 +844,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -851,9 +859,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -868,9 +874,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -879,9 +883,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ⚠️  TYPO: '20% Off' ad image says 'First Tiime Customers' — fix to 'First Time' in Canva and re-export</t>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✅  TYPO FIXED: '20% Off' ad image updated — 'First Time Customers' confirmed</t>
         </is>
       </c>
     </row>
@@ -906,9 +910,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
@@ -930,9 +932,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
@@ -954,9 +954,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -971,9 +969,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -988,9 +984,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Meta bulk upload spreadsheet column names and add Creative Type
Corrected column headers to match Meta's exact required format.
Added 'Creative type: Single image ad' column. All ads set to PAUSED.

https://claude.ai/code/session_01KqjHkizaco74VDp8DBP6wH
</commit_message>
<xml_diff>
--- a/ads-strategy/meta-bulk-upload.xlsx
+++ b/ads-strategy/meta-bulk-upload.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Ads" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instructions &amp; Checklist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="How To Upload" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,7 +29,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -39,12 +39,6 @@
       <b val="1"/>
       <color rgb="005D3A1A"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <color rgb="00000000"/>
-    </font>
-    <font>
-      <color rgb="001a7a1a"/>
     </font>
   </fonts>
   <fills count="5">
@@ -91,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -99,18 +93,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,90 +468,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="68" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="68" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ad Name</t>
+          <t>Campaign name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
+          <t>Ad set name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Ad Set Name</t>
+          <t>Ad name</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Primary Text (Body Copy)</t>
+          <t>Creative type</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Primary text</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Headline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Call To Action</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Image (upload to Meta first)</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Call to action</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Image hash</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Website URL</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="115" customHeight="1">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Display URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Parks Apparel — Relaunch 2026</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Hats — Outdoor Interest Audience</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>Yellowstone Trucker Hat — America's First NP</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Parks Apparel — Relaunch 2026</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Hats — Outdoor Interest Audience</t>
-        </is>
-      </c>
       <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Single image ad</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Old Faithful. Bison-filled valleys. America's first national park — on your head.
 Our embroidered Yellowstone National Park trucker hat is built for the trail, the road trip, and everywhere in between.
@@ -569,54 +583,64 @@
 🏔️ Shop now → parksapparel.com</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>America's First National Park On Your Head</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Embroidered Yellowstone Trucker Hat — $31.95 | 5 Colors</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>UPLOAD: Yellowstone hat ad image</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>PASTE IMAGE HASH HERE</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>https://parksapparel.com/products/embroidered-yellowstone-national-park-sign-trucker-cap</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Upload image to Meta Media Library first, then paste image hash here</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="115" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>parksapparel.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="110" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Parks Apparel — Relaunch 2026</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Tees — National Parks Fan Audience</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Protect Our Parks Big Bend — 1% Donation</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Parks Apparel — Relaunch 2026</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Tees — National Parks Fan Audience</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Single image ad</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Your purchase does more than look good.
 Parks Apparel donates 1% of every sale to the National Parks Foundation — protecting places like Big Bend for generations to come.
@@ -624,54 +648,64 @@
 Check out the Protect Our Parks Collection → parksapparel.com</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Protect What You Love</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>1% of all sales donated to the National Parks Foundation</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>UPLOAD: Protect Our Parks Big Bend ad image</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>PASTE IMAGE HASH HERE</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>https://parksapparel.com/products/protect-our-parks-big-bend-national-park-unisex-fit-soft-t-shirt</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Strong cause-marketing angle — A/B test vs identity angle</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="115" customHeight="1">
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>parksapparel.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="110" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Parks Apparel — Relaunch 2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Mugs — Outdoor Interest Audience</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>Yosemite Camp Mug — Morning Scene</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Parks Apparel — Relaunch 2026</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Mugs — Outdoor Interest Audience</t>
-        </is>
-      </c>
       <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Single image ad</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Every morning starts better with Yosemite.
 Our Yosemite National Park mug goes everywhere you do — from the campsite to the kitchen table.
@@ -679,54 +713,64 @@
 Shop now → parksapparel.com</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Start Every Morning at Yosemite</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Yosemite Mugs — Starting at $17.95 | Ships Fast</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>UPLOAD: Yosemite mug camp scene ad image</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>PASTE IMAGE HASH HERE</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>https://parksapparel.com/products/yosemite-national-park-line-art-accent-coffee-mug-11oz-15oz-blue-black-pink-red</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Confirm Instagram handle — ad shows @parksapparelcom (missing dot)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="115" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>parksapparel.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="110" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Parks Apparel — Relaunch 2026</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Mugs — Outdoor Interest Audience</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Yosemite Camp Mug — Product Shot</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Parks Apparel — Relaunch 2026</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Mugs — Outdoor Interest Audience</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Single image ad</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Half Dome. El Capitan. The Valley.
 Now in your hands every morning.
@@ -734,54 +778,64 @@
 ☕ Shop parksapparel.com</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Half Dome. El Capitan. In Your Hands.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Yosemite Enamel Camp Mug — parksapparel.com</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>UPLOAD: Yosemite camp mug product photo</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>PASTE IMAGE HASH HERE</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>https://parksapparel.com/products/yosemite-national-park-line-art-accent-coffee-mug-11oz-15oz-blue-black-pink-red</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>Clean product shot — great for cold audiences</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="115" customHeight="1">
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>parksapparel.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Parks Apparel — Relaunch 2026</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Discount — Cold Audience</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>20% Off — HappyTrails20 — New Customers</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Parks Apparel — Relaunch 2026</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Discount — Cold Audience</t>
-        </is>
-      </c>
       <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Single image ad</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>PAUSED</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>First time shopping Parks Apparel? Welcome to the parks. 🏔️
 Use code HAPPYTRAILS20 at checkout for 20% off your entire order.
@@ -789,34 +843,34 @@
 👇 Shop now → parksapparel.com</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Park Lovers Like You Get 20% Off Everything</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Use code HAPPYTRAILS20 | First-time customers only | parksapparel.com</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Use code HAPPYTRAILS20 | First-time customers only</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>UPLOAD: 20% off HappyTrails20 ad image</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>PASTE IMAGE HASH HERE</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>https://parksapparel.com</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>Typo fixed ✅ — Confirm HAPPYTRAILS20 code is active in Shopify before running</t>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>parksapparel.com</t>
         </is>
       </c>
     </row>
@@ -831,171 +885,164 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="95" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>HOW TO USE THIS FILE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>HOW TO UPLOAD TO META ADS MANAGER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>STEP 1 — Upload your 5 ad images to Meta</t>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>STEP 1 — Upload your images to Meta Media Library</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Go to Meta Ads Manager → Media Library → Upload each image</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+          <t xml:space="preserve">  In Meta Ads Manager → go to Media Library (left sidebar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upload each of your 5 ad images one by one</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>STEP 2 — Update the Image column</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  After uploading, click each image → copy the Image Hash (looks like: a1b2c3d4e5f6...)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  After uploading, copy the image hash from Meta and paste into the 'Image' column on the Ads sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>STEP 2 — Paste Image Hashes into this spreadsheet</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>STEP 3 — Fix these issues before uploading</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Replace each 'PASTE IMAGE HASH HERE' cell with the actual hash from Meta</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ✅  TYPO FIXED: '20% Off' ad image updated — 'First Time Customers' confirmed</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Match each hash to the correct ad row</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ⚠️  CHECK: Yosemite mug ad shows '@parksapparelcom' — confirm this is your correct Instagram handle</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⚠️  CONFIRM: HAPPYTRAILS20 discount code is active in Shopify (Discounts section)</t>
+          <t>STEP 3 — Import into Ads Manager</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ✅  All product URLs have been pre-filled and are live</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
+          <t xml:space="preserve">  In Ads Manager → top menu → Import → Spreadsheet Upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upload this file (.xlsx)</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>STEP 4 — Upload to Meta Ads Manager</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ads are set to PAUSED so they won't spend until you review and activate them</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  In Ads Manager → click Import → Spreadsheet → upload this file</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Meta will create all 5 ads inside your existing Advantage+ campaign</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>STEP 4 — Review and activate</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Check each ad in Ads Manager before turning on</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>PRODUCT URLS</t>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Assign each ad to the correct campaign and ad set if prompted</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Yellowstone Trucker Hat:</t>
+          <t xml:space="preserve">  Flip status from PAUSED to ACTIVE when ready</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  parksapparel.com/products/embroidered-yellowstone-national-park-sign-trucker-cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Protect Our Parks Big Bend Tee:</t>
+          <t xml:space="preserve">  • Creative type = 'Single image ad' for all 5 ads</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  parksapparel.com/products/protect-our-parks-big-bend-national-park-unisex-fit-soft-t-shirt</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Yosemite Line Art Mug:</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  parksapparel.com/products/yosemite-national-park-line-art-accent-coffee-mug-11oz-15oz-blue-black-pink-red</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Homepage (for discount ad):</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  parksapparel.com</t>
+          <t xml:space="preserve">  • Call to action = 'SHOP_NOW' for all ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Confirm HAPPYTRAILS20 discount code is active in Shopify before activating that ad</t>
         </is>
       </c>
     </row>

</xml_diff>